<commit_message>
Ehancement to synchronize the oneDrive was completed
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-con2\Documents\UiPath\AMP14_00_LiberarCalculoCoste\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP14_00_LiberarCalculoCoste\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BF46CC-7800-4C79-A9DD-1FDC89055229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140A7D6B-92D0-4CA4-8006-3572B168C778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
   <si>
     <t>Name</t>
   </si>
@@ -209,9 +209,6 @@
     <t>AMP14_00_LiberarCalculoCoste</t>
   </si>
   <si>
-    <t>saplogon.exe;EXCEL</t>
-  </si>
-  <si>
     <t>SAP_LCCostesTransaction</t>
   </si>
   <si>
@@ -243,6 +240,15 @@
   </si>
   <si>
     <t>VarianteCostoTraspaso</t>
+  </si>
+  <si>
+    <t>VM_MachingUser</t>
+  </si>
+  <si>
+    <t>Credenciales del usuario de la sesion actual</t>
+  </si>
+  <si>
+    <t>saplogon.exe;EXCEL;OneDrive</t>
   </si>
 </sst>
 </file>
@@ -342,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -353,6 +359,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -650,7 +659,7 @@
         <v>54</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>55</v>
@@ -668,9 +677,15 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
+      <c r="A7" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2946,56 +2961,56 @@
       <c r="A6" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>61</v>
+      <c r="B6" s="8" t="s">
+        <v>60</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>62</v>
+      <c r="D6" s="8" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>63</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>64</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>65</v>
+      <c r="D7" s="9" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>66</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>67</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>68</v>
+      <c r="D8" s="9" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>70</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>69</v>
+      <c r="D9" s="9" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>